<commit_message>
Verify vintage/commitment across 6 more entities; fix double-counting and citation-confidence bugs; ONT/LiquidAI/SchoolHack commitment treatment; dashboard notes + fixed column widths; PRD v1.7
</commit_message>
<xml_diff>
--- a/data/source_of_truth/Investment_Register_Intake.xlsx
+++ b/data/source_of_truth/Investment_Register_Intake.xlsx
@@ -574,15 +574,19 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Beyond Limits\2. Transaction Closure Documents\Beyond Limits - Investment Summary.docx</t>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Beyond Limits\2. Transaction Closure Documents\Beyond Limits - Note Purchase Agreement (Executed with Exhibits).pdf</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>AI-extracted from Investment Summary + Note Purchase Agreement - Series C Preferred Stock tranche. HIGH CONFIDENCE.</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from the executed Note Purchase and Investment Agreement dated January 21, 2020 between Beyond Limits, Inc. and MOZN Holding RSC Ltd (Schedule A - Schedule of Investor): the $80,000,000 Series C Preferred Stock commitment is split across 4 scheduled Stock Purchase Closings (conversion/purchase price $5.1523/share) - $30,000,000 due later of 3-month anniversary or 31 Mar 2020, $30,000,000 due later of 6-month anniversary or 30 Jun 2020, $10,000,000 due later of 9-month anniversary or 30 Sep 2020, and $10,000,000 due later of 12-month anniversary or 31 Dec 2020. Cross-checked against actual cash flow: $30M (2020-03-31), $30M (2020-06-07), $10M (2020-09-29) were paid (matching the first 3 tranches almost exactly); the 4th $10,000,000 tranche (due 31 Dec 2020) does NOT appear in the cash flow extract - i.e. genuinely undrawn, not a data gap. Committed remains $80,000,000 (the full contractual commitment); Remaining Commitment of ~$10M reflects this real undrawn tranche, not an error.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -842,15 +846,19 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\EsyaSoft\Esyasoft - Investment Summary.docx</t>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\EsyaSoft\2. Transaction Closure Documents\Executed and dated note purchase agreement.pdf</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>AI-extracted from Investment Summary: $2.5M convertible note, 10% interest, 2yr term, converts to 21% fully diluted equity. HIGH CONFIDENCE.</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from the executed Note Purchase Agreement dated 1 September 2020 between Esyasoft Holding Limited (a DIFC company) and MOZN Holding RSC Ltd: purchase price of a convertible note = $2,500,000, matching the register exactly. Referenced alongside a side letter with IHC Capital Holding LLC and a separate IHC Note Purchase Agreement dated 27 April 2020 (IHC co-invested in a related/parallel note). FLAG for follow-up: the cashflow extract records the $2,500,000 deployment on 2020-02-09 - 7 months BEFORE this agreement's stated date - not yet reconciled (possible bridge funding formalized later, or a tracker date entry issue; needs the earlier 'Esyasoft - earlier note' documents, dated around 4 Feb 2020, to resolve). Also found a SEPARATE cashflow tag 'Esyasoft Holding (Debt)' (-$411,765 on 2021-07-07, +$470,784.65 on 2022-12-07) plus a +$5,000,000 flow on 2022-05-10 under 'Esyasoft Holding' - none of these are represented by a register row yet; NOT included in this row's Committed/close_date - needs its own follow-up as a likely additional/separate tranche, not yet investigated.</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -883,7 +891,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2020-03-25</t>
+          <t>2019-04-15</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -894,15 +902,19 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Flyr\3. Monitoring\FlyR - Investment Summary.docx</t>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Flyr\2. Transaction Documents\1. Transaction Documents - Series B\FLYR - Subordinated Convertible Note Purchase Agreement 2019 0415.pdf</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>AI-extracted: $5M cash for B-1 Prefs + $5M convertible note converted to B-2 Prefs = $10M total. HIGH CONFIDENCE.</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from two executed documents: (1) Subordinated Convertible Note Purchase Agreement dated April 15, 2019 between FLYR, Inc. and MOZN Holding RSC Ltd - a $5,000,000 convertible note (cross-checked: cashflow shows $4,999,998.09 deployed 2019-04-15); (2) Series B Preferred Stock Purchase Agreement (2020) - MOZN purchased Series B-1 Preferred Stock directly for cash at $2.5710/share (cross-checked: cashflow shows $5,000,001.91 deployed 2020-03-25), AND the 2019 Note converted into Series B-2 Preferred Stock per Section 1.2(d) of the SPA. Total = $10,000,000, matching the register exactly (both cash legs sum to $10,000,000.00 to the cent). VINTAGE JUDGMENT: this is a genuine two-stage investment spanning two calendar years (first capital actually at risk 2019-04-15 via the Note; the Series B-1 direct purchase + Note conversion followed in 2020). Set close_date/vintage to the EARLIER, first-capital-deployment date (2019-04-15) per the 'vintage = year money was first put to work' convention (consistent with the HeyGears lesson: always use the earliest concrete cash-deployment evidence, not just the named round's own year) - this MOVES vintage from 2020 to 2019 versus the prior (unverified) register value. Flag for user review if a 'named round year' convention (2020, per the Series B closing) is preferred instead.</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -987,7 +999,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2019-09-30</t>
+          <t>2020-12-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -998,15 +1010,19 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Heygears\1. Due Diligence Documents\Heygears - Investment Summary.docx</t>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Heygears\2.0 Transaction Closure Documents\11. Heygears - Notice of Payment (EXE).pdf</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>AI-extracted from Investment Summary: $60M for RMB4,753,356.29 registered capital, Equity Subscription Agreement 30 Sep 2019. HIGH CONFIDENCE. NOTE: folder '4.3 New round Jun 2026' contains THIRD-PARTY term sheets (Guangzhou Industrial Investment, Zhangjiagang Mingyi Lingxing, Shanghai Wofu) raising a NEW Series C round from OTHER investors - these are NOT G42 investments and were excluded from this row.</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from the executed Closing Binder (2.0 Transaction Closure Documents): Notice of Payment (EXE) instructs MOZN Holding RSC Ltd to wire USD 60,000,000 pursuant to the Equity Subscription Agreement dated September 30, 2019, matching the register's amount exactly. Investing entity (MOZN Holding RSC Ltd) confirmed via the Notice of Payment addressee and the Closing Binder Index cover page ('Purchase of Equity Interests... By MOZN Holding RSC Ltd'). Instrument confirmed as Registered Capital (RMB 4,753,356.29) per the Equity Subscription Agreement, consistent with a China WFOE/JV capital contribution structure. VINTAGE: the SPA and all transaction documents are dated as of September 30, 2019, but the Closing Binder Index cover page states 'CLOSING DATE: JANUARY 9, 2020', and the actual USD 60,000,000 cash wire is recorded on 2020-12-01 (cross-checked against Tracker_Extract_Reconciled cashflow) - an ~11 month gap between the stated closing date and actual funding, plausibly a China outbound foreign-exchange regulatory approval delay. The tracker's own Vintage column already independently shows 2020, not 2019. USER CONFIRMED (2026-08-16): use 2020 as the vintage year (both the binder's closing date and the actual cash wire point to 2020); close_date set to the actual cash wire date 2020-12-01 as the most concrete evidence of when the investment was funded. LESSON: always cross-check contract/signing date vs. stated closing date vs. actual cash movement date - these can genuinely diverge by many months and the gap recurs across deals, don't assume the SPA date is the vintage without checking the others.</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1154,15 +1170,19 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Jysan Technologies\2. Transaction Documents\1. Final Execution Documents\1. Jysan - Investment Summary.pdf</t>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Jysan Technologies\2. Transaction Documents\1. Final Execution Documents\3. JYSAN - Subscription Agreement - Executed Version.pdf</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>AI-extracted: $20M for 7,959,497 A Ordinary Shares (3%), Subscription Agreement 6 Apr 2021. HIGH CONFIDENCE.</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from the executed Subscription Agreement dated 6 April 2021 between Jysan Technologies Ltd, the Existing Shareholder, Jysan Holding LLC, and QAZ42 Investment SPV RSC LTD (the Subscriber): fixed Purchase Price of $20,000,000 for the Subscription Shares (A Ordinary Shares), matching the register exactly. Investing entity (QAZ42 Investment SPV RSC LTD) and close date (6 April 2021) both confirmed directly from the agreement's parties clause and execution date. Cross-checked against actual cash flow: $20,000,000 paid 2021-06-16 (within the agreement's 60-day Completion window from signing), matching exactly.</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1238,7 +1258,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>66599843.43</v>
+        <v>60819862.91</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1258,15 +1278,19 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Liquid AI\1. Transaction Docs\Liquid AI - Executed Docs (G42) Nov 25\Liquid AI Inc. - Series A - G42 Side Letter [EXECUTED].pdf</t>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Liquid AI\LiquidAI_Core42 - SO2 - Execution Version (1).pdf</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>AI-extracted from executed Side Letter: Initial G42 Closing $19,999,882.40 cash (165,082 shares) + Second G42 Closing $46,599,961.03 deemed consideration (384,643 shares, satisfied via compute cluster procurement, not cash) = $66,599,843.43 total Series A Preferred. HIGH CONFIDENCE on terms; note second tranche was non-cash (compute credit), worth flagging distinctly if precision matters.</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) net of a Core42 cashback/credit: Core42 Holding US LLC's Service Order No. 2 with LiquidAI, Inc. (referencing the Series A Purchase Agreement and Side Letter, both dated 23 Dec 2024) confirms Core42 will issue an invoice for USD 40,819,980.52 upon signature - USD 35,040,000.00 is the value of compute Core42 provides, and USD 5,779,980.52 is the 'Company Balance'/'Credit' referenced in the Purchase Agreement and Side Letter. USER-CONFIRMED (2026-08-16): this credit is a cashback expected FROM Core42 (a G42 affiliate) as part of the transaction, so it is netted OUT of the Committed figure here (gross USD 66,599,843.43 - USD 5,779,980.52 credit = USD 60,819,862.91), matching the tracker's own treatment of this investment (~USD 60.82M).</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1446,7 +1470,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2500000</v>
+        <v>2750000</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1471,10 +1495,14 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>CONFIRMED from the actual Subscription Agreement, Clause 3.1: Core42 Investments 1 SPV RSC LTD subscribed 25,000 Preferred Shares for USD $2,500,000 - exact match to tracker figure. HIGH CONFIDENCE - document-verified, no longer a tracker fallback.</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from the executed Subscription Agreement (Core42 Investments 1 SPV RSC Ltd and Airev Holding Limited): Clause 4.4 - within 45 days of Completion, the Company shall enter into a cloud services agreement with an affiliate of the Investor, entitling it to a credit for cloud services worth USD 250,000 (at prevailing market rates). USER-CONFIRMED (2026-08-16): this is a real compute commitment, separate from the USD 2,500,000 cash equity subscription - total Committed = USD 2,750,000.00 (2,500,000 equity + 250,000 compute credit), matching the tracker's own figure exactly.</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1494,7 +1522,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>30000000</v>
+        <v>14999998.94</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1503,7 +1531,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2023-04-30</t>
+          <t>2023-04-12</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1514,15 +1542,19 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\TFH - Worldcoin\1. DD Docs, IAF &amp; Closing Docs\2. Investment Note - Worldcoin\IC - Note\Investment summary note - Worldcoin - Apr-23.pdf</t>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\TFH - Worldcoin\1. DD Docs, IAF &amp; Closing Docs\3. Closing Docs\TFH - Series C - Stock Purchase Agreement (Executed) (April 12_ 2023).pdf</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>AI-extracted from Investment Summary Note (Apr 2023) + Term Sheet (3 Mar 2023): G42 allocation USD 30m in Series C Preferred + Token Warrants, Tools for Humanity Corporation (Worldcoin legal entity), post-money $2.4bn. HIGH CONFIDENCE on amount. fund_vehicle_id NOT explicitly named - needs the actual SPA. RESOLVED (user 2026-08-15): WLD tokens received were exchanged for ~$100M SAR in Inveniam - see Inveniam-SAR-TBD row. WLD token holding itself remains a separate line (already sold off per earlier note). ACCOUNTING TREATMENT AGREED (2026-08-15): the $100M WLD-token exchange (14 Nov 2024, cashflow TRK-CF-EQ-0049) is tagged 'Non-Cash - Asset Exchange' in Tracker_Extract_Reconciled (ref 'WLD-Inveniam-SAR-Swap-2024'). At the POSITION level this stays as-is (a real, legitimate ~6.66x distribution/gain on the WLD token holding - user confirmed a gain was booked on the WLD tokens). It should be EXCLUDED from any future PORTFOLIO-LEVEL aggregate cash paid-in/distributed/IRR calculation, since no actual cash left or entered the fund - it funded Inveniam's SAR directly. Per-position TVPI/MOIC for both TFH and Inveniam are correct as calculated; only a future aggregate rollup needs to filter this out.</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from executed Series C Preferred Stock Purchase Agreement (TFH - Series C - Stock Purchase Agreement (Executed) (April 12, 2023).pdf), Exhibit A (Schedule of Purchasers): MOZN Holding RSC Ltd purchased 65,413 shares of Series C Preferred Stock for USD 14,999,998.94 (as an Additional Closing investor under the same April 12, 2023 Agreement). Investing entity (MOZN Holding RSC Ltd) and instrument (Series C Preferred Stock) also confirmed via the MOZN-specific signature pages (TFH - Series C - MOZN HOLDING RSC LTD.pdf) for the SPA, Amended and Restated IRA, Voting Agreement, Co-Sale Agreement, and Warrant Purchase Agreement (Token Warrant), all executed as of April 12, 2023. Cross-checked against actual cash flow: cashflow TRK-CF-EQ-0032 (investment_id 'Tools for Humanity Corporation', 2023-05-29) = USD 14,999,998.94, matching the Exhibit A figure to the cent. The tracker separately tags two small additional payments under investment_id 'WLD Tokens' (not the Series C Preferred Stock purchase): USD 5,875 (2023-05-29, TRK-CF-EQ-0033) and USD 1,000 (2023-07-07, TRK-CF-EQ-0034) - USER CONFIRMED (2026-08-16) these are the Token Warrant exercise payments to receive the WLD tokens, not fees. CORRECTS a prior shallow 'AI-extracted' estimate of USD 30,000,000 (conflated the Series C Preferred cash investment with the separately-exercised, non-cash Token Warrant - no additional cash outflow is recorded around the July 2023 Token Warrant Exercise). Vintage year (2023) is unchanged either way. RESOLVED (user 2026-08-15): WLD tokens received were exchanged for ~$100M SAR in Inveniam - see Inveniam-SAR-TBD row. WLD token holding itself remains a separate line (already sold off per earlier note). ACCOUNTING TREATMENT AGREED (2026-08-15): the $100M WLD-token exchange (14 Nov 2024, cashflow TRK-CF-EQ-0049) is tagged 'Non-Cash - Asset Exchange' in Tracker_Extract_Reconciled (ref 'WLD-Inveniam-SAR-Swap-2024'). At the POSITION level this stays as-is (a real, legitimate ~6.66x distribution/gain on the WLD token holding - user confirmed a gain was booked on the WLD tokens). It should be EXCLUDED from any future PORTFOLIO-LEVEL aggregate cash paid-in/distributed/IRR calculation, since no actual cash left or entered the fund - it funded Inveniam's SAR directly. Per-position TVPI/MOIC for both TFH and Inveniam are correct as calculated; only a future aggregate rollup needs to filter this out.</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1812,13 +1844,21 @@
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Beyond Limits\2. Transaction Closure Documents\Beyond Limits - Note Purchase Agreement (Executed with Exhibits).pdf</t>
+        </is>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>AI-extracted: $20M convertible note @ 6% p.a., converts to C Prefs. HIGH CONFIDENCE.</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from the executed Note Purchase and Investment Agreement dated January 21, 2020 (Schedule A) and the Unsecured Convertible Promissory Note itself: Beyond Limits, Inc. issued a $20,000,000 convertible promissory note to MOZN Holding RSC Ltd, 6% simple interest p.a., maturing 31 Dec 2020, converting to Series C Preferred Stock at $5.1523/share. Cross-checked against actual cash flow: $20,000,000 paid 2020-02-18, matching exactly.</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">

</xml_diff>

<commit_message>
Verify Neuralink and vTv Therapeutics against primary documents (8-K, executed SPA)
</commit_message>
<xml_diff>
--- a/data/source_of_truth/Investment_Register_Intake.xlsx
+++ b/data/source_of_truth/Investment_Register_Intake.xlsx
@@ -1386,15 +1386,19 @@
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Neuralink (Project Cortex)\Transaction Documents\Neuralink Investment Summary .docx</t>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\Neuralink (Project Cortex)\Transaction Documents\SIGNED - Neuralink SPA (Series E)_Redacted.pdf</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>AI-extracted: 990,099 Series E Preferred shares @ $50.50/share = $49,999,999.50. Side Letter/IRA dated 30 May 2025; funding due by 4 June 2025 per Payment Direction Letter. HIGH CONFIDENCE.</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from the executed Series E Preferred Stock Purchase Agreement dated 30 May 2025 between Neuralink Corp and its Series E investors: Schedule A - Schedule of Series E Investors lists Expansion Project Technologies Holding 12 SPV RSC Ltd for a Total Purchase Price of $49,999,999.50 (990,099 Series E Preferred shares @ $50.50/share), matching the register exactly. Cross-checked against actual cash flow: $49,999,999.50 paid 2025-06-04, matching exactly.</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1621,7 +1625,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>G42 Health Care AI Holding RSC Ltd</t>
+          <t>G42 Investments AI Holding RSC Ltd</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1639,7 +1643,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2022-02-18</t>
+          <t>2022-05-31</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1650,15 +1654,19 @@
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\VTVT - vTv Therapeutics\Transaction Docs\Term Sheet-vtv.pdf</t>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\VTVT - vTv Therapeutics\Transaction Docs\4. 24May\G - 8-K Body (marked).pdf</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>AI-extracted via OCR (scanned PDF): Non-binding Term Sheet - G42 Health Care AI Holding RSC Ltd to acquire 10% of vTv Therapeutics Inc. common stock for $25M ($12.5M cash at closing + $12.5M secured note due in 1 year). A separate $20M milestone payment (in equity, upon FDA approval, funded via R&amp;D expenditure not cash) is NOT included in this amount. MEDIUM CONFIDENCE: this is a NON-BINDING draft term sheet, not a signed closing document - needs the actual signed agreement to confirm final terms. close_date is the folder date (18 Feb 22), not a date stated in the document itself.</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from vTv Therapeutics Inc.'s Form 8-K (Item 1.01, public SEC filing - VTVT is Nasdaq-listed): on [April/May] 2022, vTv Therapeutics Inc. and G42 Investments AI Holding RSC Ltd entered into a Common Stock Purchase Agreement for 10,386,274 Class A common shares at ~$2.41/share, aggregate purchase price USD 25,000,000 (USD 12,500,000 cash at closing + USD 12,500,000 via a promissory note of G42 Investments due at the 1-year anniversary), matching the register's committed amount exactly. CORRECTS the investing entity from 'G42 Health Care AI Holding RSC Ltd' (carried over from an earlier non-binding term sheet) to 'G42 Investments AI Holding RSC Ltd' (the entity actually named in the signed agreement per the 8-K). Cross-checked against actual cash flow: USD 12,500,000 paid 2022-05-31 (the cash tranche - close_date set to this date since the 8-K's own draft text has the exact day redacted/marked as a redline), USD 12,031,250 paid 2023-02-28 (the note settlement, ~9 months later, slightly below USD 12,500,000 - not yet reconciled, possible negotiated discount or partial repayment). Separately, a further USD 20-30,000,000 FDA-approval-contingent Milestone Shares/Cash payment is NOT included in this USD 25,000,000 Committed figure, consistent with the existing register note. NOTE: source document is a REDLINE/COMPARISON draft of the 8-K, not the final filed version - the commercial terms match the final public filing but the exact execution date was not captured from this draft; the public EDGAR filing itself would confirm the precise date if needed.</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">

</xml_diff>

<commit_message>
Apply user-confirmed business decisions (BL cancellation, ONT), verify VTVT via public IR filing, challenge Mena Mobile currency claim, flag EsyaSoft exit as open item
</commit_message>
<xml_diff>
--- a/data/source_of_truth/Investment_Register_Intake.xlsx
+++ b/data/source_of_truth/Investment_Register_Intake.xlsx
@@ -579,7 +579,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>CONFIRMED (2026-08-16) from the executed Note Purchase and Investment Agreement dated January 21, 2020 between Beyond Limits, Inc. and MOZN Holding RSC Ltd (Schedule A - Schedule of Investor): the $80,000,000 Series C Preferred Stock commitment is split across 4 scheduled Stock Purchase Closings (conversion/purchase price $5.1523/share) - $30,000,000 due later of 3-month anniversary or 31 Mar 2020, $30,000,000 due later of 6-month anniversary or 30 Jun 2020, $10,000,000 due later of 9-month anniversary or 30 Sep 2020, and $10,000,000 due later of 12-month anniversary or 31 Dec 2020. Cross-checked against actual cash flow: $30M (2020-03-31), $30M (2020-06-07), $10M (2020-09-29) were paid (matching the first 3 tranches almost exactly); the 4th $10,000,000 tranche (due 31 Dec 2020) does NOT appear in the cash flow extract - i.e. genuinely undrawn, not a data gap. Committed remains $80,000,000 (the full contractual commitment); Remaining Commitment of ~$10M reflects this real undrawn tranche, not an error.</t>
+          <t>CONFIRMED (2026-08-16) from the executed Note Purchase and Investment Agreement dated January 21, 2020 between Beyond Limits, Inc. and MOZN Holding RSC Ltd (Schedule A - Schedule of Investor): the $80,000,000 Series C Preferred Stock commitment is split across 4 scheduled Stock Purchase Closings (conversion/purchase price $5.1523/share) - $30,000,000 due later of 3-month anniversary or 31 Mar 2020, $30,000,000 due later of 6-month anniversary or 30 Jun 2020, $10,000,000 due later of 9-month anniversary or 30 Sep 2020, and $10,000,000 due later of 12-month anniversary or 31 Dec 2020. Cross-checked against actual cash flow: $30M (2020-03-31), $30M (2020-06-07), $10M (2020-09-29) were paid (matching the first 3 tranches almost exactly); the 4th $10,000,000 tranche (due 31 Dec 2020) does NOT appear in the cash flow extract - i.e. genuinely undrawn, not a data gap. Committed remains $80,000,000 (the full contractual commitment); Remaining Commitment of ~$10M reflects this real undrawn tranche, not an error. CANCELLED (user-confirmed 2026-08-16): the final ~$10,000,000 Series C tranche (due 31 Dec 2020 per Schedule A) will not be drawn - substantial time has passed with no intent to invest further. No cancellation document on file yet (user is trying to obtain one) - dashboard Committed is pinned to Invested to reflect this (see _COMMITTED_EQUALS_INVESTED_DEALS in live_exited_sections.py).</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>CONFIRMED (2026-08-16) from the executed Note Purchase Agreement dated 1 September 2020 between Esyasoft Holding Limited (a DIFC company) and MOZN Holding RSC Ltd: purchase price of a convertible note = $2,500,000, matching the register exactly. Referenced alongside a side letter with IHC Capital Holding LLC and a separate IHC Note Purchase Agreement dated 27 April 2020 (IHC co-invested in a related/parallel note). FLAG for follow-up: the cashflow extract records the $2,500,000 deployment on 2020-02-09 - 7 months BEFORE this agreement's stated date - not yet reconciled (possible bridge funding formalized later, or a tracker date entry issue; needs the earlier 'Esyasoft - earlier note' documents, dated around 4 Feb 2020, to resolve). Also found a SEPARATE cashflow tag 'Esyasoft Holding (Debt)' (-$411,765 on 2021-07-07, +$470,784.65 on 2022-12-07) plus a +$5,000,000 flow on 2022-05-10 under 'Esyasoft Holding' - none of these are represented by a register row yet; NOT included in this row's Committed/close_date - needs its own follow-up as a likely additional/separate tranche, not yet investigated.</t>
+          <t>CONFIRMED (2026-08-16) from the executed Note Purchase Agreement dated 1 September 2020 between Esyasoft Holding Limited (a DIFC company) and MOZN Holding RSC Ltd: purchase price of a convertible note = $2,500,000, matching the register exactly. Referenced alongside a side letter with IHC Capital Holding LLC and a separate IHC Note Purchase Agreement dated 27 April 2020 (IHC co-invested in a related/parallel note). FLAG for follow-up: the cashflow extract records the $2,500,000 deployment on 2020-02-09 - 7 months BEFORE this agreement's stated date - not yet reconciled (possible bridge funding formalized later, or a tracker date entry issue; needs the earlier 'Esyasoft - earlier note' documents, dated around 4 Feb 2020, to resolve). Also found a SEPARATE cashflow tag 'Esyasoft Holding (Debt)' (-$411,765 on 2021-07-07, +$470,784.65 on 2022-12-07) plus a +$5,000,000 flow on 2022-05-10 under 'Esyasoft Holding' - none of these are represented by a register row yet; NOT included in this row's Committed/close_date - needs its own follow-up as a likely additional/separate tranche, not yet investigated. OPEN ITEM - USER FLAGGED (2026-08-16): user recalls investing $2,500,000 (matches this row) and believes the position has since EXITED at approximately 2x - consistent with a +$5,000,000 cash flow already observed on 2022-05-10 under 'Esyasoft Holding' (exactly 2x $2,500,000), which is currently NOT reflected in this row's lifecycle_state (still 'Live'). User will provide further details - do not change lifecycle_state or Distributions until confirmed with a document/the tracker's own classification.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>CONFIRMED from the actual FINAL executed Series D Purchase Agreement + its Disclosure Schedule (folder '4. 28 Oct 24'): Expansion Project Technologies Holding 7 SPV RSC Ltd (the 'Initial Purchaser') paid $19,999,998.17 cash for 6,925,351 Series D shares, plus a $20,947,397.27 Convertible Promissory Note converting into 7,253,404 further shares = $40,947,395.44 total. HIGH CONFIDENCE - document-verified, no longer based on a non-binding draft term sheet. close_date set to 28 Oct 2024 per the final docs folder.</t>
+          <t>CONFIRMED from the actual FINAL executed Series D Purchase Agreement + its Disclosure Schedule (folder '4. 28 Oct 24'): Expansion Project Technologies Holding 7 SPV RSC Ltd (the 'Initial Purchaser') paid $19,999,998.17 cash for 6,925,351 Series D shares, plus a $20,947,397.27 Convertible Promissory Note converting into 7,253,404 further shares = $40,947,395.44 total. HIGH CONFIDENCE - document-verified, no longer based on a non-binding draft term sheet. close_date set to 28 Oct 2024 per the final docs folder. USER CLARIFICATION (2026-08-16): the structure is a $20,000,000 initial convertible note investment, which on conversion added a further ~$20,000,000 cash investment PLUS accrued interest paid in kind as additional shares (not cash) - actual CASH invested is $40,000,000; the additional ~$947,395.44 in the Committed/Invested figures represents the value of the PIK interest shares received, not further cash deployed.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -1334,15 +1334,19 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\MenaMobile\1. Due Diligence Documents\Mena Mobile - Investment Summary.docx</t>
+          <t>C:\Users\divyesh.mahajan\OneDrive - G42\Desktop\0.1 SPPM ###\1. I N V E S T M E N T S  -  Global (Ex China)\0. E Q U I T Y\MenaMobile\2. Transaction Closure Documents\A-1 MOZN - Mena - Series B - SPA (execution version).pdf</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>AI-extracted: $8M for 21,419,829 Series B Preferred Shares, Agreement dated 29 Jul 2019. HIGH CONFIDENCE.</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
+          <t>CONFIRMED (2026-08-16) from the executed Series B Preferred Share Purchase Agreement dated 29 July 2019 between Mena Mobile Inc. and MOZN Holding RSC Ltd: Schedule II (Share Purchase Information) states explicitly 'MOZN Holding RSC Ltd | 21,419,829 Series B Preferred Shares | Per Share Price US$0.373486 | Purchase Price US$8,000,000' - CURRENCY VERIFIED AS USD, not AED. USER QUERY (2026-08-16): user recalled this might be AED 8,000,000 - checked directly against the signed SPA's own Schedule II, which states the amount in US$ explicitly, not AED. Keeping USD 8,000,000 - if further evidence of an AED-denominated commitment surfaces, revisit.</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1659,7 +1663,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>CONFIRMED (2026-08-16) from vTv Therapeutics Inc.'s Form 8-K (Item 1.01, public SEC filing - VTVT is Nasdaq-listed): on [April/May] 2022, vTv Therapeutics Inc. and G42 Investments AI Holding RSC Ltd entered into a Common Stock Purchase Agreement for 10,386,274 Class A common shares at ~$2.41/share, aggregate purchase price USD 25,000,000 (USD 12,500,000 cash at closing + USD 12,500,000 via a promissory note of G42 Investments due at the 1-year anniversary), matching the register's committed amount exactly. CORRECTS the investing entity from 'G42 Health Care AI Holding RSC Ltd' (carried over from an earlier non-binding term sheet) to 'G42 Investments AI Holding RSC Ltd' (the entity actually named in the signed agreement per the 8-K). Cross-checked against actual cash flow: USD 12,500,000 paid 2022-05-31 (the cash tranche - close_date set to this date since the 8-K's own draft text has the exact day redacted/marked as a redline), USD 12,031,250 paid 2023-02-28 (the note settlement, ~9 months later, slightly below USD 12,500,000 - not yet reconciled, possible negotiated discount or partial repayment). Separately, a further USD 20-30,000,000 FDA-approval-contingent Milestone Shares/Cash payment is NOT included in this USD 25,000,000 Committed figure, consistent with the existing register note. NOTE: source document is a REDLINE/COMPARISON draft of the 8-K, not the final filed version - the commercial terms match the final public filing but the exact execution date was not captured from this draft; the public EDGAR filing itself would confirm the precise date if needed.</t>
+          <t>CONFIRMED (2026-08-16) from vTv Therapeutics' public press release (ir.vtvtherapeutics.com, 1 June 2022, 'vTv Therapeutics Announces Investment by and Entry into Collaboration and License Agreement with affiliates of G42 Healthcare') and Form 8-K: $25,000,000 investment by G42 Investments AI Holding RSC Ltd for 10,386,274 Class A Common shares at $2.407/share - USD 12,500,000 paid in cash at closing, remaining USD 12,500,000 payable 31 May 2023. Close date 2022-05-31 confirmed (cash closing date; the deferred payment's exact 1-year due date of 31 May 2023 corroborates this). CORRECTS the FDA-approval-contingent Milestone figure from USD 20,000,000 (an early draft 8-K redline value) to USD 30,000,000 in additional Class A shares (or cash in lieu) - per the final public press release - still NOT included in this USD 25,000,000 Committed figure. Investing entity 'G42 Investments AI Holding RSC Ltd' independently confirmed via this public source (matches the 8-K). OPEN ITEM - USER FLAGGED (2026-08-16): user recalls a possible legal/transaction fee refund that may reduce the effective net commitment (mentioned a $15,000,000 figure, unconfirmed) - NOT found in the press release, 8-K, or cash flow reviewed so far; Committed is kept at the document-verified USD 25,000,000 pending further evidence. Do not change to any other figure without a document.</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard QA pass: fix IRR convergence bug, rework number formatting, correct fund commitment figures, add fund-CAS cashflow primacy mechanism
</commit_message>
<xml_diff>
--- a/data/source_of_truth/Investment_Register_Intake.xlsx
+++ b/data/source_of_truth/Investment_Register_Intake.xlsx
@@ -2259,10 +2259,14 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>CONFIRMED from Capital Call Notice #1 (21 Jun 2019): Total Capital Commitment USD 300,000,000 (100%), Limited Partner is 'Galbot Holding RSC Ltd' (a G42 SPV) per the Subscription Agreement and A&amp;R LPA. First drawdown was only 1% ($3M). close_date approximated to 18 Jun 2019 (fee period start date referenced in the notice). HIGH CONFIDENCE on commitment amount and vehicle name. NOTE: folder contains a '3. Liquidation FY25' subfolder - possible wind-down in progress, not yet investigated.</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr"/>
+          <t>CONFIRMED from Capital Call Notice #1 (21 Jun 2019): Total Capital Commitment USD 300,000,000 (100%), Limited Partner is 'Galbot Holding RSC Ltd' (a G42 SPV) per the Subscription Agreement and A&amp;R LPA. First drawdown was only 1% ($3M). close_date approximated to 18 Jun 2019 (fee period start date referenced in the notice). HIGH CONFIDENCE on commitment amount and vehicle name. NOTE: folder contains a '3. Liquidation FY25' subfolder - possible wind-down in progress, not yet investigated. UPDATED 2026-08-18: found and read the executed Side Letter dated December 2023 (effective 1 Jan 2023) - the General Partner irrevocably waived the Investor's entire outstanding/uncalled Capital Contribution obligation of US$217,693,608. The $300,000,000 figure remains the correct ORIGINAL subscription commitment (unchanged, still primary-source-confirmed for that date), but no further capital will ever be called - the dashboard's Committed figure is now pinned to Invested via _COMMITTED_EQUALS_INVESTED_DEALS (see live_exited_sections.py) to reflect this.</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2286,7 +2290,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>50000000</v>
+        <v>17112500</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2307,10 +2311,14 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>CONFIRMED from executed CEF (15 Nov 2021) + Anchor MOU Terms: LP commitment of the lesser of 50% of aggregate LP commitments or $50M in Acies Ventures Fund I, L.P. (target fund size $150M), via G42 Investments AI Holding RSC Ltd. ADDITIONAL RIGHT not reflected in this $ figure: G42/Mozn is also an economic assignee entitled to 9.9% of the GP's carried interest - a separate, non-capital economic interest not captured as a register row. HIGH CONFIDENCE on the $50M LP commitment.</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr"/>
+          <t>UPDATED 2026-08-18: the Q1 2026 Capital Account Statement (G42 Investments AI Holding RSC Limited, period ended 31 Mar 2026) explicitly states 'Commitment $17,112,500' (Paid-in Capital $15,726,388, Remaining $1,386,113) - this is the actual final/subscribed commitment, not the $50M figure. CORRECTED from the earlier CEF (15 Nov 2021) + Anchor MOU Terms citation, which described a FORMULA/CAP ('the lesser of 50% of aggregate LP commitments or $50M in Acies Ventures Fund I, L.P., target fund size $150M') rather than the actual final subscribed amount - the fund's actual size ended up smaller than the $150M target, so 50% of aggregate LP commitments landed at $17,112,500 rather than hitting the $50M cap. User flagged 2026-08-18 that the dashboard's $50M didn't match the tracker - confirmed via the CAS. HIGH CONFIDENCE (primary capital account statement, matches the tracker). ADDITIONAL RIGHT not reflected in this $ figure: G42/Mozn is also an economic assignee entitled to 9.9% of the GP's carried interest - a separate, non-capital economic interest not captured as a register row.</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard checkpoint: Overview polish + Portfolio tab restyle; add style guide
- Overview: scope tabs beside title, 3D section boxes, non-truncating KPI box,
  IB/SEC grounding note, Gross MOIC (TVPI), dashboard-wide terminology sweep
- Portfolio tab (renamed from 'Current month'): pill nav tabs, wider layout,
  darker subtotals, light-green entity rows, one-line filter actions, new as-of header
- Docs: docs/implementation/Dashboard_Style_Guide.md + PRD_CHANGELOG v1.17.0
- Checkpoint also captures in-progress legal-KB and accounts-team parity artifacts

Note: figures on the Portfolio dashboard (NAV-tab + CAS basis) do not yet
triangulate with the Overview (Live report-tab basis) - reconciliation pending.
</commit_message>
<xml_diff>
--- a/data/source_of_truth/Investment_Register_Intake.xlsx
+++ b/data/source_of_truth/Investment_Register_Intake.xlsx
@@ -8206,7 +8206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8253,28 +8253,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1. New Space Capital Fund</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>NewSpace-ICEYE-2020</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>NEEDS FOLLOW-UP</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>CONFIRMED from signed Side Letter + Drawdown 1 Notice (3 Sep 2020): New Space Capital Fund I is an SPV-style vehicle with a separate 'Sub-Fund' per deal - this is the ICEYE Oy sub-fund only (1,591,574 Series C preferred shares, 6.1% of ICEYE, EUR18,798,671.27 + fees = EUR19,015,957.27 total commitment, fully drawn at this single Drawdown 1). HIGH CONFIDENCE for THIS sub-fund. NEEDS FOLLOW-UP DOCUMENT: 20 total drawdown notices exist through 2025 in this fund's folder, indicating MULTIPLE additional sub-fund deals beyond ICEYE (tracker shows ~$36M total paid-in across 23 cashflow rows, far more than this one EUR19M sub-fund) - not yet individually identified/recorded.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>